<commit_message>
test(extraction): add test cases EXTRACT-001..010
New EXTRACT sheet in docs/test-cases.xlsx tracks 10 acceptance test cases for the entity extraction feature (phone/email/url/otp/credit-card regex + LLM smart-scan for address/name/date/bank account).

Per project policy, test cases are written before implementation so each TDD task can reference its TC-ID.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="EXTTOK" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="EXTRACT" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +26,21 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDDDDD"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +55,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1311,4 +1324,505 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Verified by</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="60" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>EXTRACT-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Share message with phone+email → entity sheet, 2 rows, both copy</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>User logged in; Flutter app installed on Android+iOS</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1. From any chat, long-press a msg "Call 0912345678 or email tan@x.com"
+2. Share → DraftRight
+3. Tap copy on phone row
+4. Tap copy on email row</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Entity sheet renders 2 group cards (Phone, Email); SnackBar "Phone copied" / "Email copied"; clipboard contains correct value</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>entity_extractor_test.dart + manual</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>EXTRACT-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Share message with no entities → tone picker shows (regression)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>User logged in</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>1. Share prose "Hello, hope you are well."
+2. Observe screen</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Tone picker renders; entity sheet never mounts</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>share_rewrite_screen_test.dart + manual</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>EXTRACT-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Smart scan adds Vietnamese address</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>User logged in; AI provider configured</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>1. Share msg containing "Địa chỉ 123 Lê Lợi Q1"
+2. Tap ✨ Smart scan</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>After spinner: 🏠 Address row appears with display "123 Lê Lợi Q1"; button hides</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>extraction.service.spec.ts + manual</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>EXTRACT-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Smart scan offline → snackbar, regex results intact</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>User logged in; device airplane mode</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>1. Airplane mode
+2. Share msg with phone+address
+3. Tap ✨ Smart scan</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>SnackBar "Smart scan unavailable"; phone row still visible &amp; copyable; Smart scan button re-enabled</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>entity_sheet_screen_test.dart + manual</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>EXTRACT-005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Card number masked on render, full value copied</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>User logged in</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>1. Share msg "Card 4242 4242 4242 4242"
+2. Observe display
+3. Long-press to reveal
+4. Tap copy</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Display shows "**** **** **** 4242"; long-press reveals full; copy yields "4242424242424242"</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>credit_card_detector_test.dart + manual</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>EXTRACT-006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>OTP detected only when trigger word present</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>User logged in</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>1. Share msg "Năm 2024 là năm tốt."
+2. Share msg "OTP 482917"</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Msg #1: empty (no trigger). Msg #2: 🔢 OTP row with 482917</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>otp_detector_test.dart + manual</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>EXTRACT-007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Long message (5000 chars) → regex &lt; 50ms, no UI freeze</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>User logged in</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>1. Share a 5000-char text containing 10 phones + 5 emails
+2. Observe load</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Sheet renders within 100ms; no jank; all 15 rows visible</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>manual perf test</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>EXTRACT-008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>iOS share extension same flow</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>User logged in on iOS device</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>1. On iOS, share msg from Notes / Messages app via share sheet
+2. Pick DraftRight</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Same entity sheet renders as Android</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>manual on iOS device</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>EXTRACT-009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Quota exceeded → 402 snackbar, regex results stay</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>User logged in; free tier quota exhausted</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>1. Share msg with phone+address
+2. Tap ✨ Smart scan</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>SnackBar "Smart scan limit reached"; phone row still visible</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>extraction_api_test.dart + manual</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>EXTRACT-010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Vietnamese diacritics + emoji in source → offsets correct</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>User logged in</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>1. Share msg "Gọi 0912345678 nhé 😊"
+2. Verify entity selection highlights</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Phone row shows; copy yields "+84912345678"; no offset crash; UTF-16 surrogates handled</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>entity_extractor_test.dart + manual</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
test(keepalive): add KEEPALIVE-001..010 (retroactive — should have landed before code)
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="EXTTOK" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="EXTRACT" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="KEEPALIVE" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1825,4 +1826,511 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Verified by</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="70" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Toggle ON installs launchd agent + sets RunAtLoad=true</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>macOS app installed, fresh state (no existing keepalive plist)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1. Launch DraftRight
+2. Open Settings &gt; General
+3. Toggle "Launch at Login" ON
+4. Run: launchctl print gui/$(id -u)/com.draftright.app.v2.keepalive</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Plist file exists at ~/Library/LaunchAgents/com.draftright.app.v2.keepalive.plist; launchctl reports state=running; RunAtLoad=true; pid set</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>KeepAliveAgent smoke test + manual</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="70" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Toggle OFF uninstalls launchd agent entirely</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Agent currently installed (toggle ON)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>1. Open Settings &gt; General
+2. Toggle "Launch at Login" OFF
+3. Run: launchctl print gui/$(id -u)/com.draftright.app.v2.keepalive</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>launchctl errors with "Could not find service"; plist file removed from ~/Library/LaunchAgents/</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="70" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>SIGKILL respawns app within 15 s when toggle ON</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Toggle ON, app running</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>1. pgrep DraftRight to get PID
+2. kill -9 &lt;pid&gt;
+3. Wait 15 s
+4. pgrep DraftRight</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>New PID found, different from original; app appears in menu bar; log shows "MONITOR Mode: HOTKEY" on startup</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="70" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Clean Quit (status 0) does NOT respawn</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Toggle ON, app running</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>1. Click menu bar icon &gt; Quit DraftRight
+2. Wait 20 s
+3. pgrep DraftRight</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>No process found. Agent honors SuccessfulExit=false guard — clean exits stay quit.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="70" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Reconcile updates plist path when app is moved</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>App installed at /Applications/DraftRight.app, toggle ON, agent installed</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>1. Quit app
+2. mv /Applications/DraftRight.app ~/Downloads/DraftRight.app
+3. Launch from ~/Downloads/
+4. cat plist | grep ProgramArguments</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Plist ProgramArguments[0] now points to ~/Downloads/DraftRight.app/Contents/MacOS/DraftRight (not /Applications). Self-healing works.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="70" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Boot at login when toggle ON</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Toggle ON, app quit</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>1. Log out
+2. Log back in
+3. Within 30 s, pgrep DraftRight</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>App launched automatically by launchd; menu bar icon visible.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="70" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>No respawn loop on repeated immediate crash</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Hypothetical broken build that crashes on startup</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>1. Replace DraftRight binary with one that exits 1 immediately
+2. Launch via launchd
+3. Observe /tmp/draftright-keepalive.err</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>launchctl reports throttling — agent does not respawn more often than every 10 s (ThrottleInterval guard).</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>manual (load-time only)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="70" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>First-launch reconcile installs agent if missing</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Toggle ON in UserDefaults but plist file deleted manually</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>1. Quit app
+2. rm ~/Library/LaunchAgents/com.draftright.app.v2.keepalive.plist
+3. Launch app
+4. ls ~/Library/LaunchAgents/</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Plist recreated by AppModel.init reconcile call.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="70" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Toggle is idempotent — multiple ON taps do not double-load</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Toggle ON, agent loaded</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>1. Toggle OFF then ON ten times
+2. launchctl list | grep keepalive</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Exactly one launchd job; no zombie duplicates.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="70" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>OS-initiated termination respawns app</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Toggle ON, app running. Simulate OS kill (e.g. RunningBoard memory pressure).</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>1. sudo launchctl kickstart -k gui/$(id -u)/com.draftright.app.v2.keepalive</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>App respawned by launchd. Models real-world OOM/sleep-cycle terminations.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
test(keepalive): add KEEPALIVE-WIN-001..010 (Windows port test cases)
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -10,6 +10,7 @@
     <sheet name="EXTTOK" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="EXTRACT" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="KEEPALIVE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="KEEPALIVE-WIN" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2333,4 +2334,510 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Verified by</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="70" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-WIN-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Toggle ON creates Scheduled Task with logon trigger + RestartOnFailure</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Fresh Windows install, no prior "DraftRight Keep Alive" task</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1. Launch DraftRightWindows.exe
+2. Open Settings &gt; Launch at Login
+3. Toggle ON
+4. Run in PowerShell: Get-ScheduledTask -TaskName "DraftRight Keep Alive"</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Task exists, State=Ready; LogonTrigger.Enabled=$true; Settings.RestartOnFailure.Interval=PT10S, Count=10</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>manual on Windows</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="70" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-WIN-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Toggle OFF deletes the Scheduled Task</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Task currently installed</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>1. Settings &gt; toggle "Launch at Login" OFF
+2. Get-ScheduledTask -TaskName "DraftRight Keep Alive"</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>PowerShell errors with "No MSFT_ScheduledTask objects found". Task XML backup also deleted from %LOCALAPPDATA%\DraftRight\keepalive.xml.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>manual on Windows</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="70" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-WIN-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Force-kill respawns app within ~15 s</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Toggle ON, app running</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>1. Get-Process DraftRightWindows | %{$_.Id}
+2. Stop-Process -Id &lt;pid&gt; -Force
+3. Wait 15 s
+4. Get-Process DraftRightWindows</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>New PID found, app back in tray. RestartOnFailure trigger fired.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>manual on Windows</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="70" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-WIN-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Clean Exit does NOT respawn</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Toggle ON, app running</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>1. Right-click tray icon &gt; Quit
+2. Wait 20 s
+3. Get-Process DraftRightWindows</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>No process. RestartOnFailure only fires on non-zero exit; menu Quit returns 0.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>manual on Windows</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="70" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-WIN-005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Reconcile refreshes task XML when exe is moved</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>App installed at C:\Program Files\DraftRight\, task registered</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>1. Quit app
+2. Copy folder to C:\Users\&lt;user&gt;\AppData\Local\Programs\DraftRight\
+3. Run from new location
+4. Get-ScheduledTask "DraftRight Keep Alive" | Export-ScheduledTask | Select-String "&lt;Command&gt;"</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Task XML now contains the new path. Self-heal via IsPathFresh check.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>manual on Windows</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="70" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-WIN-006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Boot at logon when toggle ON</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Toggle ON, app quit</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>1. Sign out
+2. Sign back in
+3. Within 30 s, Get-Process DraftRightWindows</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>App running with PID. LogonTrigger fired during sign-in.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>manual on Windows</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="70" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-WIN-007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Independent of legacy HKCU\...\Run key</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Toggle ON, both registry "Run" and Scheduled Task present</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>1. reg delete "HKCU\Software\Microsoft\Windows\CurrentVersion\Run" /v DraftRight /f
+2. Sign out + back in</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>App still launches at logon (via the Scheduled Task, even though the Run key is gone). The two paths are intentionally independent.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>manual on Windows</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="70" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-WIN-008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Task is per-user (LeastPrivilege, no UAC prompt)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Toggle ON during app run as Standard User (no admin elevation)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>1. Sign in as a standard (non-admin) user
+2. Launch DraftRight
+3. Toggle "Launch at Login" ON</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Task created without a UAC prompt. RunLevel=LeastPrivilege, LogonType=InteractiveToken.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>manual on Windows</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="70" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-WIN-009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Toggle idempotent — multiple ON taps do not create duplicates</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Toggle ON, agent installed</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>1. Toggle OFF then ON ten times
+2. Get-ScheduledTask -TaskPath \ | Where-Object TaskName -eq "DraftRight Keep Alive"</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Exactly one task. schtasks /Create /F overwrites rather than duplicating.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>manual on Windows</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="70" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>KEEPALIVE-WIN-010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Battery-allowed and no-network-required</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Toggle ON, laptop on battery, no internet</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>1. Disconnect Wi-Fi + unplug laptop
+2. Stop-Process DraftRightWindows -Force
+3. Wait 15 s</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>App respawns. DisallowStartIfOnBatteries=false + StopIfGoingOnBatteries=false + RunOnlyIfNetworkAvailable=false guarantees offline coverage.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>manual on Windows</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
test(keyboard): add KEYBOARD-MULTI-001..054 (before-code mandate)
Seed 54 test cases for Tier β multi-language Android keyboard into
docs/test-cases.xlsx via openpyxl. Groups: Telex composition (16),
Telex backspace (5), edge cases (4), layout swap (7), globe key (3),
long-press accent picker (5), space-bar label (1), settings
persistence (3), backward compatibility (4), plus tones (6).

Spec: docs/superpowers/specs/2026-05-17-android-multilang-keyboard-design.md
Plan: docs/superpowers/plans/2026-05-17-android-multilang-keyboard.md

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -11,6 +11,7 @@
     <sheet name="EXTRACT" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="KEEPALIVE" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="KEEPALIVE-WIN" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="KEYBOARD-MULTI" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2840,4 +2841,2338 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H55"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Verified by</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="50" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Telex aa → â</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Type a,a</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits â</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="50" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Telex oo → ô</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Type o,o</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ô</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="50" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Telex ee → ê</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Type e,e</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ê</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Telex ow → ơ</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Type o,w</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ơ</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Telex uw → ư</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Type u,w</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ư</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="50" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Telex aw → ă</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Type a,w</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ă</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="50" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Telex dd → đ</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Type d,d</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits đ</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="50" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Telex aaj → ậ</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Type a,a,j</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ậ (â + dot)</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="50" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Telex uow → ươ</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Type u,o,w</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ươ</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Telex uowj → ượ</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Type u,o,w,j</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ượ</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Telex case preserved on shift</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>VI active, shift on</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Type A,A</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits Â</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Telex no-op for non-rule keys</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Type q</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Direct commit q (no composing)</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="50" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Telex a+s → á</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Type a,s</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits á</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="50" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Telex a+f → à</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Type a,f</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits à</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="50" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Telex a+r → ả</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Type a,r</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ả</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="50" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Telex a+x → ã</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Type a,x</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ã</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="50" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Telex a+j → ạ</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Type a,j</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ạ</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="50" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-018</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Telex aaj sequence applies tone after circumflex</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Type a,a,j</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ậ</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="50" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Type "việt"</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Type v,i,e,t,j</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Field shows việt</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="50" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-020</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Type "chương"</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Type c,h,u,o,w,n,g</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Field shows chương</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="50" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Type "người"</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Type n,g,u,o,w,i,f</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Field shows người</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="50" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Type "tiếng"</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Type t,i,e,s,n,g</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Field shows tiếng</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="50" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Backspace un-composes one step</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>VI active, "việt" composed</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Press ⌫</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Field shows việ (last char un-composed via composer)</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="50" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-024</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Backspace at empty composer passes through</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>VI active, no composing state</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Press ⌫</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>InputConnection.deleteSurroundingText called</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="50" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Backspace removes mark before vowel</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>VI active, "â" composed</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Press ⌫</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Field shows a (â un-composed)</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="50" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Backspace clears tone before mark</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>VI active, "ậ" composed</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Press ⌫</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Field shows â (tone removed)</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="50" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Multiple backspaces clear composer state</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>VI active, "việt" composed</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Press ⌫ four times</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Composer state empty; further ⌫ deletes via IC</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="50" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-028</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Non-letter mid-cluster commits pending</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>VI active, "vie" composing</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Type space</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Field shows "vie " (vowel cluster committed)</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="50" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Language switch mid-cluster commits + resets</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>VI active, "vie" composing</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Tap globe to switch to EN</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Composing region committed as "vie"; composer.reset() called</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardControllerTest.kt</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="50" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-030</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Paste mid-cluster clears composer</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>VI active, "vie" composing</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>System paste fires commitText</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Composer onStartInput-like reset; pasted text intact</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardControllerTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="50" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Composing length cap at 32 chars</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Type 33 vowel keys</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits at length 32; new key starts fresh</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTest.kt</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="50" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>EN baseline unchanged</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>EN active</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Type "hello"</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Identical keystroke output to today (regression)</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>EnglishLanguagePackTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="50" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>AZERTY French layout</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>FR active</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Tap QWERTY position of "a"</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Letter "a" emitted (AZERTY puts a in QWERTY-q slot)</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>FrenchLanguagePackTest.kt</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="50" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-034</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Spanish ñ key</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>ES active</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Tap ñ key</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Field shows ñ</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>SpanishLanguagePackTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="50" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>German QWERTZ layout</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>DE active</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Tap QWERTY position of "z"</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Letter "z" emitted (QWERTZ y/z swapped)</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>GermanLanguagePackTest.kt</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="50" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-036</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>German ß key</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>DE active</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Tap ß key</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Field shows ß</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>GermanLanguagePackTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="50" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Portuguese ç key</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>PT active</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Tap ç key</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Field shows ç</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>PortugueseLanguagePackTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="50" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-038</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Language cycle order = VI &gt; FR &gt; ES &gt; DE &gt; IT &gt; PT</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>All enabled</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Tap globe 6 times</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Cycles through VI, FR, ES, DE, IT, PT, back to start</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardControllerTest.kt</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="50" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-039</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Globe tap cycles enabled languages</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>VI + EN enabled</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Tap globe</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>activeLanguageId flips between VI and EN</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardControllerTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="50" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-040</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Globe long-press opens IME picker</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Long-press globe 500ms</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>InputMethodManager.showInputMethodPicker() called</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardControllerTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="50" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-041</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Single enabled language: globe tap is no-op</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Only EN enabled</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Tap globe</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>activeLanguageId unchanged; strip not shown</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardControllerTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="50" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-042</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Long-press a in ES shows á à ä â ã</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>ES active</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Hold a key 300ms</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>AccentPopupView appears above key with 5 options + a</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>AccentPopupViewTest + manual</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="50" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Long-press ñ in ES: no popup</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>ES active</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Hold ñ key</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>No popup (ñ not in accents map); short-press commits ñ</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>SpanishLanguagePackTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="50" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-044</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Long-press a in FR shows é è ê variants for e key</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>FR active</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Hold e key</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Popup with é è ê ë</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>FrenchLanguagePackTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="50" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-045</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Finger up without drag = short-press</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>ES active</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Hold a, release before drag</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Plain a committed; popup dismisses</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>AccentPopupViewTest + manual</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="50" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-046</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Drag selects + release commits</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>ES active</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Hold a, drag right, release on á</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Field shows á</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="50" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-047</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Space bar shows current language displayName</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Look at space bar</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Reads "Tiếng Việt" (or current.displayName)</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>manual on emulator</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="50" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-048</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>activeLanguageId survives Force-Stop</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Force-stop app; relaunch IME</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>VI still active</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardControllerTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="50" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-049</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>enabledLanguageIds reorder persists</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>VI &gt; EN order saved</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Reorder to EN &gt; VI in Settings; relaunch</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Globe cycles EN &gt; VI in new order</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>manual on emulator</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="50" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-050</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Disabling all languages forces EN</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>User disables all</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Open keyboard</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>EN forced; activeLanguageId="en"; toast/log warning</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardControllerTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="50" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-051</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>EN-only users see no behavior change</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Fresh install, no setting changes</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Type "hello world"</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Output identical to pre-Tier-β</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>EnglishLanguagePackTest.kt + manual</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="50" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-052</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Existing tone toolbar still functions</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Type text, tap "Polished"</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Tone rewrite flow unchanged</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>manual + integration</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="50" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-053</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Share intent unchanged</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>EN active</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Long-press text → Share → DraftRight</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Share rewrite flow unchanged</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="50" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-054</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>/rewrite payload includes only text + tone (no inputLanguage)</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Tap Polished</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Backend request body has text + tone only</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>BackendClient inspection</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
test(windows): add SINGLE-INST-001..006 (before-code mandate)
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -12,6 +12,7 @@
     <sheet name="KEEPALIVE" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="KEEPALIVE-WIN" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="KEYBOARD-MULTI" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="SINGLE-INST" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5175,4 +5176,322 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Verified by</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="50" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SINGLE-INST-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>First launch starts normally</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>No DraftRight.exe running</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Launch DraftRight.exe</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Single tray icon appears; single DraftRight.exe in Task Manager</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Manual on Windows 11 x64</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="50" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SINGLE-INST-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Second launch exits silently</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>One DraftRight.exe already running with tray icon</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Launch DraftRight.exe a second time</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Second process exits immediately; still exactly one tray icon; still one DraftRight.exe in Task Manager</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Manual on Windows 11 x64</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="50" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SINGLE-INST-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>No duplicate taskbar icon when RewritePanel is open</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>DraftRight running, rewrite panel open via hotkey</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Launch DraftRight.exe a second time</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Taskbar still shows exactly one DraftRight entry; no flicker</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Manual on Windows 11 x64</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SINGLE-INST-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Mutex released on graceful exit</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>DraftRight running</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Quit via tray menu → Exit; wait 2s; launch DraftRight.exe again</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>New process launches normally; tray icon reappears</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Manual on Windows 11 x64</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SINGLE-INST-005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Mutex released on process kill</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>DraftRight running</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Task Manager → End Task on DraftRight.exe; wait 2s; launch DraftRight.exe</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>New process launches normally (kernel reclaims the abandoned mutex)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Manual on Windows 11 x64</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="50" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>SINGLE-INST-006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Different Windows users can each run their own instance</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>User A signed in with DraftRight running</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Fast-switch to User B; launch DraftRight.exe as User B</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>User B's instance runs (Mutex is Local\, not Global\); both users have their own tray icon</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Manual on Windows 11 x64 multi-user host</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
test(ios): add KEYBOARD-MULTI-IOS-001..056 (before-code mandate)
Mirrors the Android KEYBOARD-MULTI sheet with iOS-specific
adjustments per the 2026-05-18 evening plan revision:

- Globe-key tests (039-041) reflect iOS reality: DraftRight does
  NOT intercept the system globe key. In-keyboard language cycle
  uses swipe-right/left on space bar instead.
- TC-027 (Empty-buffer backspace) and TC-028 (Space mid-cluster)
  encode the three composer-routing fixes that emerged on Android.
- TC-055 (Full Access OFF) confirms typing works offline; only
  the rewrite needs the network privilege.
- TC-056 (memory < 50 MB) tracks Apple's keyboard-ext memory cap.

56 rows total. Verifies via 'Verified by' column → Swift test
files that will be created in Stages 1-9 of the plan.
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -13,6 +13,7 @@
     <sheet name="KEEPALIVE-WIN" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="KEYBOARD-MULTI" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="SINGLE-INST" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="KEYBOARD-MULTI-IOS" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5494,4 +5495,2422 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H57"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Verified by</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="50" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Telex aa → â</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Type a,a</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits â</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="50" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Telex oo → ô</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Type o,o</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ô</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="50" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Telex ee → ê</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Type e,e</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ê</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="50" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Telex ow → ơ</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Type o,w</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ơ</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="50" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Telex uw → ư</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Type u,w</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ư</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="50" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Telex aw → ă</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Type a,w</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ă</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="50" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Telex dd → đ</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Type d,d</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits đ</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="50" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Telex aaj → ậ</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Type a,a,j</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ậ (â + dot)</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="50" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Telex uow → ươ</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Type u,o,w</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ươ</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Telex uowj → ượ</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Type u,o,w,j</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ượ</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Telex case preserved on shift</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>VI active, shift on</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Type A,A</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits Â</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="50" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Telex no-op for non-rule keys</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Type q</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Direct insertText q (no marked text)</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="50" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Telex a+s → á</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Type a,s</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits á</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="50" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Telex a+f → à</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Type a,f</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits à</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="50" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Telex a+r → ả</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Type a,r</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ả</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="50" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Telex a+x → ã</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Type a,x</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ã</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="50" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Telex a+j → ạ</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Type a,j</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ạ</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="50" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-018</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Telex aaj sequence applies tone after circumflex</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Type a,a,j</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits ậ</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="50" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Type "việt"</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Type v,i,e,t,j</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Field shows việt</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="50" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-020</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Type "chương"</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Type c,h,u,o,w,n,g</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Field shows chương</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="50" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Type "người"</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Type n,g,u,o,w,i,f</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Field shows người</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="50" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Type "tiếng"</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Type t,i,e,s,n,g</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Field shows tiếng</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="50" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-023</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Backspace un-composes one step</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>VI active, "việt" composed</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Press ⌫</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Field shows việ (marked text updated via setMarkedText)</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="50" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-024</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Backspace from empty buffer falls back to deleteBackward</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>VI active, no composing state</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Press ⌫</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>textDocumentProxy.deleteBackward called</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="50" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Backspace removes mark before vowel</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>VI active, "â" composed</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Press ⌫</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Field shows a (â un-composed via stripOneLayer)</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="50" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-026</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Backspace clears tone before mark</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>VI active, "ậ" composed</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Press ⌫</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Field shows â (tone removed)</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="50" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-027</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Empty-buffer backspace calls unmarkText explicitly</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>VI active, single char "v" composed</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Press ⌫</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>textDocumentProxy.unmarkText fires + field clears (no stuck marked region)</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardViewControllerTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="50" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-028</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Space mid-cluster commits pending via composer</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>VI active, "vie" composing</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Press space</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Field shows "vie " (vowel cluster committed THEN space appended — not replaced)</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardViewControllerTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="50" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-029</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Language swipe mid-cluster commits + resets</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>VI active, "vie" composing</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Swipe right on space bar</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Composing region committed as "vie"; composer.reset() called</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardViewControllerTests.swift</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="50" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-030</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Paste mid-cluster clears composer</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>VI active, "vie" composing</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>System paste fires</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Composer reset on next key; pasted text intact</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardViewControllerTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="50" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-031</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Composing length cap at 32 chars</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Type 33 vowel keys</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Composer commits at length 32; new key starts fresh</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>TelexComposerTests.swift</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="50" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-032</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>EN baseline unchanged</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>EN active</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Type "hello"</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Identical keystroke output to pre-Tier-β iOS keyboard (regression)</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>EnglishLanguagePackTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="50" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-033</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>AZERTY French layout</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>FR active</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Tap QWERTY position of "a"</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Letter "a" emitted (AZERTY puts a in QWERTY-q slot)</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>FrenchLanguagePackTests.swift</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="50" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-034</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Spanish ñ key</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>ES active</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Tap ñ key</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Field shows ñ</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>SpanishLanguagePackTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="50" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-035</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>German QWERTZ layout</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>DE active</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Tap QWERTY position of "z"</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Letter "z" emitted (QWERTZ y/z swapped)</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>GermanLanguagePackTests.swift</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="50" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-036</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>German ß key</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>DE active</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Tap ß key</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Field shows ß</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>GermanLanguagePackTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="50" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-037</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Portuguese ç key</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>PT active</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Tap ç key</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Field shows ç</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>PortugueseLanguagePackTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="50" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-038</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Language cycle order = VI &gt; FR &gt; ES &gt; DE &gt; IT &gt; PT (Tan's preference, matches Android)</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>All enabled</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Swipe right on space 6 times</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Cycles through VI, FR, ES, DE, IT, PT, back to start</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardControllerTests.swift</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="50" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-039</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Swipe-right on space-bar cycles enabled languages</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>VI + EN enabled</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Swipe right on space bar (&gt;80 px)</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>activeLanguageId advances; space-bar label updates</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardViewControllerTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="50" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-040</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>System iOS globe key opens system keyboard picker (we DO NOT intercept)</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Tap iOS system globe key (bottom-left)</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>iOS native picker / next system keyboard — DraftRight does NOT handle</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Manual on iPhone</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="50" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-041</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Single enabled language: swipe-space is no-op</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Only EN enabled</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Swipe right on space bar</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Nothing happens; tap on space still emits space</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardViewControllerTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="50" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-042</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Long-press a in ES shows á à ä â ã</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>ES active</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Hold a key 400ms</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>AccentPopupView appears above key with 5 options + a</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>AccentPopupViewTests + manual</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="50" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-043</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Long-press ñ in ES: no popup</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>ES active</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Hold ñ key</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>No popup (ñ not in accents map); short-press commits ñ</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>SpanishLanguagePackTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="50" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-044</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Long-press e in FR shows é è ê ë variants</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>FR active</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Hold e key</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Popup with é è ê ë</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>FrenchLanguagePackTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="50" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-045</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Finger up without drag = short-press</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>ES active</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Hold a, release before drag</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Plain a committed; popup dismisses</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>AccentPopupViewTests + manual</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="50" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-046</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Drag selects + release commits via UIPanGestureRecognizer</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>ES active</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Hold a, drag right, release on á</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Field shows á</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="50" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-047</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Space bar shows current language displayName</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Look at space bar</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Reads "Tiếng Việt" (or current.displayName)</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Manual on iPhone</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="50" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-048</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>activeLanguageId survives keyboard re-bind</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Switch to another keyboard then back to DraftRight</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>VI still active</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardControllerTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="50" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-049</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>enabledLanguageIds reorder persists across App Group</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>VI &gt; EN order saved in Flutter app</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Reorder to EN &gt; VI in Settings; relaunch keyboard ext</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Swipe-space cycles in new order</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Manual on iPhone</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="50" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-050</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Disabling all languages forces EN</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>User disables all</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Open keyboard</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>EN forced; activeLanguageId="en"; no crash</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>KeyboardControllerTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="50" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-051</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>EN-only users see no behavior change</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>Fresh install, no setting changes</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Type "hello world"</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Output identical to pre-Tier-β iOS keyboard</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>EnglishLanguagePackTests.swift + manual</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="50" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-052</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Existing tone toolbar still functions</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Type text, tap "Polished"</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Tone rewrite flow unchanged; replaceAllText calls unmarkText FIRST</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Manual + integration</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="50" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-053</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Share extension unchanged</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>EN active</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Long-press text → Share → DraftRight</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Share rewrite flow unchanged</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="50" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-054</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>/rewrite payload includes only text + tone (no inputLanguage)</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>VI active</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Tap Polished</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Backend request body has text + tone only</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>BackendClient inspection</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="50" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-055</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Full Access disabled → typing works, rewrite shows banner</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>Allow Full Access OFF for DraftRight Keyboard in iOS Settings</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Open keyboard, type, tap tone button</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Typing works locally (Telex composer is offline). Rewrite shows 'Allow Full Access in Settings' banner — no network call attempted.</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Manual on iPhone 14/SE</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="50" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>KEYBOARD-MULTI-IOS-056</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Memory under 50 MB with all 7 packs loaded</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>All 7 enabledLanguageIds</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Type one sentence in each language; observe Xcode Allocations</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Peak ext memory &lt; 50 MB (Apple cap ≈ 70 MB)</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Xcode Instruments + manual</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: add SECFIX test cases for critical review fixes
Test cases SECFIX-001..006 covering Windows auto-login removal,
Linux sign-out, and website verify-email redirect validation.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -14,6 +14,7 @@
     <sheet name="KEYBOARD-MULTI" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="SINGLE-INST" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="KEYBOARD-MULTI-IOS" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="SECFIX" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7913,4 +7914,318 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Verified by</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SECFIX-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Windows: no auto-login with test credentials on fresh launch</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Fresh Windows install, no saved session (delete auth.json)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1. Launch DraftRightWindows.exe
+2. Watch backend logs / network for POST /auth/login</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>No login request fires automatically; app stays logged out until user logs in via Settings; AutoLoginAsync no longer exists in App.cs</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Code inspection + manual on Windows 11</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SECFIX-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Linux: sign-out clears session without crash</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Linux app running, user logged in</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1. Open app menu
+2. Click Sign Out</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Session cleared (auth.json tokens removed), UI returns to logged-out state, no AttributeError in stderr</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>manual on Linux + python -m py_compile</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SECFIX-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Website: verify-email rejects cross-origin next param</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Valid pending verification token</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1. Open /verify-email?token=&lt;valid&gt;&amp;next=https://evil.com
+2. Complete verification</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Browser redirected to /account (fallback), NOT evil.com</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>redirect helper unit check + manual</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SECFIX-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Website: verify-email honors safe same-origin next param</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Valid pending verification token</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1. Open /verify-email?token=&lt;valid&gt;&amp;next=/checkout?plan=pro
+2. Complete verification</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Browser redirected to /checkout?plan=pro</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SECFIX-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Website: verify-email without next shows success UI</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Valid pending verification token</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1. Open /verify-email?token=&lt;valid&gt; (no next param)
+2. Complete verification</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Success screen rendered, no redirect</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SECFIX-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Website: verify-email rejects protocol-relative and backslash next</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Valid pending verification token</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1. Try next=//evil.com
+2. Try next=/\evil.com</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Both redirect to /account fallback</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>redirect helper unit check</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix(website): harden safeNextPath against URL-renormalization bypass (#17)
String prefix checks miss next=/\t/evil.com — the browser strips the
tab and navigates to //evil.com. Reject \t\n\r outright, then resolve
next against our own origin via the URL parser and require an unchanged
origin with no credentials, returning a path-only string.

Verified against 11 vectors incl. /\t/evil.com, /\t//evil.com, /\evil.com.
TC: SECFIX-007

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -7922,7 +7922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8225,6 +8225,50 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SECFIX-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Website: verify-email rejects whitespace-obfuscated next (tab/newline strip bypass)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Valid pending verification token</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1. Try next=/\t/evil.com
+2. Try next=/\t//evil.com
+3. Try next=/path with embedded CR/LF</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>All resolve to /account fallback (browser would strip tab/newline making //evil.com); safeNextPath returns null on any \t\n\r</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>redirect helper logic test (11 vectors, ALL PASS)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test: add VOICE test cases (VOICE-001..012) for keyboard voice input
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -15,6 +15,7 @@
     <sheet name="SINGLE-INST" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="KEYBOARD-MULTI-IOS" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="SECFIX" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="VOICE" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -8272,4 +8273,564 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Verified by</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>VOICE-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Node: input_kind=speech prepends speech preamble</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>resolvePrompt-equivalent called with tone=polished, input_kind=speech</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Prompt = SPEECH_PREAMBLE + polished tone prompt</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>rewrite.service.spec.ts: 'speech input_kind prepends preamble'</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>VOICE-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Node: absent/typed input_kind = unchanged prompt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>POST /rewrite without input_kind and with input_kind=typed</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Prompt identical to today; both requests 201</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>rewrite.service.spec.ts: 'typed/absent leaves prompt unchanged'</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>VOICE-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Node: invalid input_kind rejected 400</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>POST /rewrite input_kind=banana</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>400, message: input_kind must be one of the following values: typed, speech</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>DTO validation via e2e/validation spec</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>VOICE-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Go parity: same three behaviors as VOICE-001..003 byte-identical</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Node running</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>shadowdiff fixtures rewrite_input_kind_speech / _typed / _invalid</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Gate rows PASS (Node/Go identical)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>shadowdiff fixtures</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>VOICE-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kotlin: InputKind enum apiValue</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>InputKind.SPEECH.apiValue</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>"speech"; TYPED → "typed"</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>InputKindTest.kt</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>VOICE-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>VoiceSession: happy path EN</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>fake recognizer returns final transcript</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>start → partial → final → polish success</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>state IDLE→LISTENING→PROCESSING→IDLE; commitResult(polished)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>VoiceSessionControllerTest.kt happy path</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>VOICE-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>VoiceSession: polish failure commits RAW transcript</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>fake recognizer ok, fake client fails (401/timeout/quota)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>start → final → polish error</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>commitResult(raw transcript) + hint banner; NEVER empty commit</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>VoiceSessionControllerTest.kt fallback tests</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>VOICE-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>VoiceSession: cancel inserts nothing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>fake recognizer</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>start → cancel while LISTENING</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>state → IDLE, no commit call</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>VoiceSessionControllerTest.kt cancel</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>VOICE-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Long-press mic = raw mode, no AI call</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>fake recognizer</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>long-press → speak → final</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>commitResult(raw), backend client NOT invoked</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>VoiceSessionControllerTest.kt raw mode</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>VOICE-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>sttLocale per pack</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>EnglishPack.sttLocale / VietnamesePack.sttLocale / JapanesePack.sttLocale</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>en-US / vi-VN / null (mic hidden for JA)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>LanguagePackSttLocaleTest.kt</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>VOICE-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Permission trampoline grant/deny</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>fresh install, RECORD_AUDIO not granted</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>tap mic → trampoline → grant; repeat with deny</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>grant: listening starts; deny: stays IDLE, key remains, re-tap re-explains</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>manual on A52</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>VOICE-012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Manual E2E vi-VN on A52</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>A52, VI pack active, logged in</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>mic → speak Vietnamese with fillers → observe</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>polished Vietnamese committed; fillers/punctuation fixed</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>manual on A52</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
test(docs): add VOICE-013/014 test cases for app-switch cancel + denied-permission guidance
VOICE-013 covers the new onFinishInput/onWindowHidden cancel (app/field
switch mid-dictation must not hot-mic or commit into the wrong field).
VOICE-014 covers the denied-permission banner added to onWindowShown's
resume-on-grant flow.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -8281,7 +8281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8830,6 +8830,90 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>VOICE-013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>App switch mid-dictation cancels session</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>dictation LISTENING or PROCESSING</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>start dictation, switch app/field</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>recognizer stops, nothing committed to new field</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>manual on A52</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>VOICE-014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Permanently denied permission shows guidance</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>RECORD_AUDIO permanently denied</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>tap mic with permission permanently denied</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>banner pointing to system settings, no dead tap</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(payment): native PayPal recurring subscriptions (backend)
PayPal as a native subscription strategy alongside LemonSqueezy/VietQR (Model A):
OAuth2 client-credentials, /v1/billing/subscriptions checkout, webhook-signature
verify, cancel via API. Webhook events → completePayment / extendByStoreRef /
cancel / expire with StoreType.PAYPAL. No hardcoding (brand via appName(), hosts
as constants, plan prices from /plans). Adds paypal_webhook_id + plan-id columns
to app_settings (idempotent SQL migration) + paypal-create-plans ops script.

Backend implemented in a prior session (see HANDOVER-2026-07-21-paypal.md);
verified this session: tsc clean, jest 174/174 green (47/47 payment). Method
stays DISABLED until enabled + configured; sandbox E2E still gated on PayPal creds.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -16,6 +16,7 @@
     <sheet name="KEYBOARD-MULTI-IOS" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="SECFIX" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="VOICE" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="PAYPAL" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -62,12 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1333,6 +1335,912 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Verified by</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PAYPAL-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>OAuth2 access token fetched via client_credentials + cached</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>paypal_client_id/secret set</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Call getAccessToken twice within token TTL</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1st call POSTs /v1/oauth2/token with Basic auth; 2nd returns cached token, no 2nd network call</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>paypal.strategy.spec.ts</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PAYPAL-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>createCheckout (monthly) uses monthly plan + returns approve URL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>paypal creds + paypal_plan_monthly set; payment.plan billing_period=monthly</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Call createCheckout</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>POST /v1/billing/subscriptions body has plan_id=monthly, custom_id=reference_code; returns links[rel=approve].href as redirect_url</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>paypal.strategy.spec.ts</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PAYPAL-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>createCheckout (yearly) uses yearly plan id</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>paypal_plan_yearly set; plan billing_period=yearly</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Call createCheckout</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>plan_id sent = yearly plan id</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>paypal.strategy.spec.ts</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PAYPAL-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>createCheckout without configured plan id → clear config error</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>paypal_plan_monthly empty</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Call createCheckout monthly</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Throws "No PayPal billing plan configured for monthly billing…"; no subscription created</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>paypal.strategy.spec.ts</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PAYPAL-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>createCheckout without credentials → not-configured error</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>paypal_client_id empty</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Call createCheckout</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Throws "PayPal is not configured…"</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>paypal.strategy.spec.ts</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PAYPAL-006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Webhook with FAILURE verification → 400 rejected</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>paypal_webhook_id set; verify API returns verification_status=FAILURE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>POST /payment/webhook/paypal with tampered body</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>verifyWebhook throws BadRequestException (400); no subscription mutated</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>paypal.strategy.spec.ts</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PAYPAL-007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Webhook with unset webhook_id → ignored (no crash)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>paypal_webhook_id empty</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>POST webhook</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Returns {type:ignored}; 200; nothing mutated</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>paypal.strategy.spec.ts</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PAYPAL-008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ACTIVATED → first-cycle activation completes pending payment + stamps store_ref</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>pending Payment exists for reference_code; verify=SUCCESS</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>POST BILLING.SUBSCRIPTION.ACTIVATED with resource.custom_id=ref, resource.id=sub</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Payment completed; subscription granted; stampStoreRef(ref, StoreType.PAYPAL, subId) called</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>payment.service.spec.ts</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PAYPAL-009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PAYMENT.SALE.COMPLETED (renewal) extends expiry via store-ref</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>active PayPal sub exists (store_ref=subId); no pending payment</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>POST PAYMENT.SALE.COMPLETED with billing_agreement_id=subId</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>fetchNextBillingUnix read; extendByStoreRef(StoreType.PAYPAL, subId, nextBilling) called</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>payment.service.spec.ts</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PAYPAL-010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>First-cycle SALE.COMPLETED after ACTIVATED does not double-grant</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ACTIVATED already completed the pending payment</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>POST PAYMENT.SALE.COMPLETED for same sub</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No new subscription row; extend to same next_billing_time is a no-op (idempotent)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>payment.service.spec.ts</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PAYPAL-011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CANCELLED webhook → cancelByStoreRef, access kept until period end</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>active PayPal sub</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>POST BILLING.SUBSCRIPTION.CANCELLED resource.id=subId</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>cancelByStoreRef(StoreType.PAYPAL, subId); status=cancelled; expires_at unchanged</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>payment.service.spec.ts</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PAYPAL-012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>EXPIRED/SUSPENDED webhook → expireByStoreRef, access revoked</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>active PayPal sub</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>POST BILLING.SUBSCRIPTION.EXPIRED resource.id=subId</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>expireByStoreRef(StoreType.PAYPAL, subId); access revoked immediately</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>payment.service.spec.ts</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>PAYPAL-013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PAYMENT.FAILED webhook → user emailed, access NOT revoked</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>active PayPal sub with user email</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>POST BILLING.SUBSCRIPTION.PAYMENT.FAILED resource.id=subId</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>sendPaymentFailed emailed; subscription NOT expired (dunning window)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>payment.service.spec.ts</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PAYPAL-014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>cancelActiveSubscription (store_type=paypal) cancels via API, keeps expires_at</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>user has active paypal sub with store_transaction_id</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>POST /payment/subscription (DELETE) as user</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>PayPal cancel API POSTed; returns {cancelled:true, expires_at unchanged}</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>payment.service.spec.ts + manual sandbox</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PAYPAL-015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>paypal method disabled until enabled → checkout 400</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>payment_methods_enabled excludes paypal</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>POST /payment/checkout method=paypal</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>404/400 "Payment method paypal is not enabled" (safe default pre-credentials)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>payment.service.spec.ts</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PAYPAL-016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>enabled-methods validation accepts paypal (has strategy)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Save payment_methods_enabled="lemonsqueezy,vietqr,paypal"</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Accepted; paypal recognized as registered method</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>payment.service.spec.ts</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PAYPAL-017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>sandbox vs live base URL selected by paypal_mode</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>paypal_mode=live</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Any API call</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>baseUrl = https://api-m.paypal.com (sandbox → api-m.sandbox.paypal.com)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>paypal.strategy.spec.ts</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PAYPAL-018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>VND plan not offered via PayPal (USD only)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>user on VND plan</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Attempt paypal checkout for VND plan</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>No paypal_plan mapping for VND → config error / VND excluded from PayPal in UI</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>manual + paypal.strategy.spec.ts</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PAYPAL-019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>tsc --noEmit + npm test green after wiring</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>feature branch</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>npx tsc --noEmit; npm test</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>No type errors; all paypal specs pass</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>CI/local</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PAYPAL-020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>E2E sandbox: checkout → approve → ACTIVATED activates Pro → cancel</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>sandbox creds + billing plans + buyer sandbox account</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Full flow in sandbox</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Subscription approved; webhook activates Pro; in-app cancel keeps access to period end</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>manual sandbox on testing server</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(#207): feed n-gram context to suggestions (phase 2a)
refreshCandidates() hardcoded previousTokens = emptyList(), leaving
TrigramCandidateEngine's next-word prediction + bigram boost as dead code.
Wire it: read the committed words before the cursor and pass them as context.

- New PreviousTokens helper — pure, shared by every language pack (not VI):
  extracts up to MAX whitespace tokens before the cursor, excludes the live
  composing word (divergence-safe suffix strip), trims attached punctuation.
- READ_LOOKBACK const bounds the getTextBeforeCursor read per keystroke.
- Unit-tested (PreviousTokensTest 7/0). Engine paths already covered by
  TrigramCandidateEngineTest.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -22,6 +22,7 @@
     <sheet name="RWCACHE" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="DIFFGRAM" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="KBD-FEEDBACK" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="KBD-VI-SUGGEST" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5258,20 +5259,309 @@
           <t>Space -&gt; spacebar sound</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Press space</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>kindOf(space)=SPACE -&gt; FX_KEYPRESS_SPACEBAR</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>KeyFeedbackTest (unit)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>KBD-FEEDBACK-3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Backspace -&gt; delete sound</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Press backspace</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>kindOf(BACKSPACE)=DELETE -&gt; FX_KEYPRESS_DELETE</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>KeyFeedbackTest (unit)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>KBD-FEEDBACK-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Enter/other keys mapped, nothing falls silent</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Press enter, shift, layer, globe</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ENTER-&gt;FX_KEYPRESS_RETURN; shift/layer/globe-&gt;OTHER-&gt;FX_KEYPRESS_STANDARD; every kind has a sound</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>KeyFeedbackTest (unit)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>KBD-FEEDBACK-5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Haptic + sound fire on device, respecting OS settings</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Physical device, System touch-sound + haptic ON</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Type letters/space/backspace; then turn OS touch-sound OFF and retype</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Buzz + click on every press; with touch-sound OFF the click is silent (OS-gated) but haptic remains per system haptic setting</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>On-device manual</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>KBD-FEEDBACK-6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Backspace auto-repeat feedback</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Physical device</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Hold backspace to auto-repeat delete</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>A feedback tick fires on each repeat delete, not just the first</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>On-device manual</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Verified by</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>VISUG-1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>previousTokens extracts committed words before cursor</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>textBeforeCursor="xin chào ", composing=""</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>returns [xin, chào] (order preserved, most-recent last)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PreviousTokensTest (unit)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>VISUG-2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>composing word is excluded from previousTokens</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Press space</t>
+          <t>textBeforeCursor="tôi là sinh viên", composing="viên"</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>kindOf(space)=SPACE -&gt; FX_KEYPRESS_SPACEBAR</t>
+          <t>strips composing suffix -&gt; [tôi, là, sinh]; caps preserved</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>KeyFeedbackTest (unit)</t>
+          <t>PreviousTokensTest (unit)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -5288,33 +5578,33 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>KBD-FEEDBACK-3</t>
+          <t>VISUG-3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Backspace -&gt; delete sound</t>
+          <t>depth capped at MAX (trigram context)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Press backspace</t>
+          <t>5 committed words</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>kindOf(BACKSPACE)=DELETE -&gt; FX_KEYPRESS_DELETE</t>
+          <t>returns only last MAX tokens</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>KeyFeedbackTest (unit)</t>
+          <t>PreviousTokensTest (unit)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -5326,33 +5616,33 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>KBD-FEEDBACK-4</t>
+          <t>VISUG-4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Enter/other keys mapped, nothing falls silent</t>
+          <t>punctuation + blank handling</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Press enter, shift, layer, globe</t>
+          <t>"Chào," / empty / all-spaces</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ENTER-&gt;FX_KEYPRESS_RETURN; shift/layer/globe-&gt;OTHER-&gt;FX_KEYPRESS_STANDARD; every kind has a sound</t>
+          <t>trailing punctuation trimmed per token; empty input -&gt; []</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>KeyFeedbackTest (unit)</t>
+          <t>PreviousTokensTest (unit)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -5364,27 +5654,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>KBD-FEEDBACK-5</t>
+          <t>VISUG-5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Haptic + sound fire on device, respecting OS settings</t>
+          <t>bigram next-word surfaces after space (on-device)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Physical device, System touch-sound + haptic ON</t>
+          <t>VI Telex pack, bigram data present</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Type letters/space/backspace; then turn OS touch-sound OFF and retype</t>
+          <t>type "xin" then space</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Buzz + click on every press; with touch-sound OFF the click is silent (OS-gated) but haptic remains per system haptic setting</t>
+          <t>candidate bar offers likely successor (e.g. chào)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -5406,37 +5696,33 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>KBD-FEEDBACK-6</t>
+          <t>VISUG-6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Backspace auto-repeat feedback</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Physical device</t>
-        </is>
-      </c>
+          <t>bigram threaded through resolver fallback</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Hold backspace to auto-repeat delete</t>
+          <t>load bundled VI pack</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>A feedback tick fires on each repeat delete, not just the first</t>
+          <t>engine has non-empty bigram heads (log: bigram heads&gt;0)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>On-device manual</t>
+          <t>WordListLoader/Resolver test</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">

</xml_diff>

<commit_message>
feat(#208): Samsung-style number-only keypad for OTP/numeric fields
Numeric fields (OTP/PIN/phone) opened the ?123 symbols layer — digits plus
@#$%&-_+() and punctuation. Samsung shows a clean number-only pad. Add a
dedicated numeric keypad and route numeric fields to it instead of reusing
symbols1.

- QwertyLayout.numericRows: single source, 3-col grid (1-9, ABC 0 back enter).
  Language-neutral, so every pack shares it via a LanguagePack.numericRows
  default getter (Rule #1) — no per-pack copy.
- QwertyKeyboardView: LAYER_NUMERIC layer; setNumericLayer() points at it
  (was symbols1). ABC escapes back to letters so the user is never trapped.
- Unit-tested (NumericLayoutTest 4/0): all digits present, char keys are
  digits-only, specials limited to ABC/backspace/enter, no space.

iOS port tracked in #209.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -23,6 +23,7 @@
     <sheet name="DIFFGRAM" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="KBD-FEEDBACK" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="KBD-VI-SUGGEST" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="KBD-NUMPAD" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5510,20 +5511,303 @@
           <t>previousTokens extracts committed words before cursor</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>textBeforeCursor="xin chào ", composing=""</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>returns [xin, chào] (order preserved, most-recent last)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PreviousTokensTest (unit)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>VISUG-2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>composing word is excluded from previousTokens</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>textBeforeCursor="tôi là sinh viên", composing="viên"</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>strips composing suffix -&gt; [tôi, là, sinh]; caps preserved</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>PreviousTokensTest (unit)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>VISUG-3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>depth capped at MAX (trigram context)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>5 committed words</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>returns only last MAX tokens</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PreviousTokensTest (unit)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>VISUG-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>punctuation + blank handling</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>"Chào," / empty / all-spaces</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>trailing punctuation trimmed per token; empty input -&gt; []</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PreviousTokensTest (unit)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>VISUG-5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>bigram next-word surfaces after space (on-device)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>VI Telex pack, bigram data present</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>type "xin" then space</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>candidate bar offers likely successor (e.g. chào)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>On-device manual</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>VISUG-6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>bigram threaded through resolver fallback</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>load bundled VI pack</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>engine has non-empty bigram heads (log: bigram heads&gt;0)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>WordListLoader/Resolver test</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Verified by</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NUMPAD-1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>All ten digits present on numeric pad</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>textBeforeCursor="xin chào ", composing=""</t>
+          <t>inspect QwertyLayout.numericRows</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>returns [xin, chào] (order preserved, most-recent last)</t>
+          <t>digits 0-9 all present</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>PreviousTokensTest (unit)</t>
+          <t>NumericLayoutTest (unit)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -5540,28 +5824,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VISUG-2</t>
+          <t>NUMPAD-2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>composing word is excluded from previousTokens</t>
+          <t>No letters/symbols on numeric pad</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>textBeforeCursor="tôi là sinh viên", composing="viên"</t>
+          <t>inspect char keys</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>strips composing suffix -&gt; [tôi, là, sinh]; caps preserved</t>
+          <t>every char key is a digit; no letters/punctuation</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>PreviousTokensTest (unit)</t>
+          <t>NumericLayoutTest (unit)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -5578,33 +5862,33 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>VISUG-3</t>
+          <t>NUMPAD-3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>depth capped at MAX (trigram context)</t>
+          <t>Only ABC/backspace/enter specials; no space</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5 committed words</t>
+          <t>inspect special keys</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>returns only last MAX tokens</t>
+          <t>specials subset {ABC,BACKSPACE,ENTER}; ABC+backspace present; no space key</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>PreviousTokensTest (unit)</t>
+          <t>NumericLayoutTest (unit)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -5616,33 +5900,37 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>VISUG-4</t>
+          <t>NUMPAD-4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>punctuation + blank handling</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>OTP field opens number-only keypad (on-device)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>real OTP/PIN field (e.g. VNeID, or numberPassword field)</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>"Chào," / empty / all-spaces</t>
+          <t>focus an OTP field with DraftRight keyboard</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>trailing punctuation trimmed per token; empty input -&gt; []</t>
+          <t>shows 3-col digit grid (1-9, ABC 0 back enter); NOT the ?123 symbols layer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>PreviousTokensTest (unit)</t>
+          <t>On-device manual</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -5654,27 +5942,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>VISUG-5</t>
+          <t>NUMPAD-5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>bigram next-word surfaces after space (on-device)</t>
+          <t>ABC escapes back to letters</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>VI Telex pack, bigram data present</t>
+          <t>numeric field focused</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>type "xin" then space</t>
+          <t>tap ABC on numeric pad</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>candidate bar offers likely successor (e.g. chào)</t>
+          <t>returns to alpha QWERTY layer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -5684,48 +5972,10 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
-        <is>
-          <t>Tan</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>VISUG-6</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>bigram threaded through resolver fallback</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>load bundled VI pack</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>engine has non-empty bigram heads (log: bigram heads&gt;0)</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>WordListLoader/Resolver test</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
         <is>
           <t>Tan</t>
         </is>

</xml_diff>

<commit_message>
feat(#207): Vietnamese typo tolerance — fuzzy candidate top-up (gap #3)
Samsung tolerates small typos; DraftRight required exact Telex. Add edit-distance
correction to the candidate bar: when the exact prefix scan leaves empty slots,
top them up with dictionary words within 1 edit of the composing buffer, so a
mistyped word still offers the right correction to tap.

- LanguageWordList.fuzzyMatches — bounded Levenshtein scan; interface default is
  empty so an mmap 50k store opts in rather than scanning every row. InMemoryWordList
  (the bootstrap path) implements it.
- TrigramCandidateEngine tops up ONLY the empty slots (exact.size < limit), so a
  correctly-typed word's exact matches are never displaced by a fuzzy guess.
  MAX_EDITS=1 keeps corrections tight on the small bootstrap dictionary.
- Conservative: surfaces corrections to tap, no aggressive auto-replace.
- Generalises to every Latin pack (en/fr/es/de/it/pt), not VI-only.

TrigramFuzzyTest 5/0; engine regression 6/0.
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -24,6 +24,7 @@
     <sheet name="KBD-FEEDBACK" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="KBD-VI-SUGGEST" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="KBD-NUMPAD" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="KBD-VI-AUTOCORRECT" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -5794,20 +5795,271 @@
           <t>All ten digits present on numeric pad</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>inspect QwertyLayout.numericRows</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>digits 0-9 all present</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>NumericLayoutTest (unit)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NUMPAD-2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>No letters/symbols on numeric pad</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>inspect char keys</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>every char key is a digit; no letters/punctuation</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>NumericLayoutTest (unit)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NUMPAD-3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Only ABC/backspace/enter specials; no space</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>inspect special keys</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>specials subset {ABC,BACKSPACE,ENTER}; ABC+backspace present; no space key</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>NumericLayoutTest (unit)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>NUMPAD-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>OTP field opens number-only keypad (on-device)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>real OTP/PIN field (e.g. VNeID, or numberPassword field)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>focus an OTP field with DraftRight keyboard</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>shows 3-col digit grid (1-9, ABC 0 back enter); NOT the ?123 symbols layer</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>On-device manual</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>NUMPAD-5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ABC escapes back to letters</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>numeric field focused</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>tap ABC on numeric pad</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>returns to alpha QWERTY layer</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>On-device manual</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Verified by</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>VIAC-1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Substitution typo surfaces correction</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>inspect QwertyLayout.numericRows</t>
+          <t>composing=nqon</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>digits 0-9 all present</t>
+          <t>candidate bar contains ngon (edit dist 1)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>NumericLayoutTest (unit)</t>
+          <t>TrigramFuzzyTest</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -5824,28 +6076,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NUMPAD-2</t>
+          <t>VIAC-2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>No letters/symbols on numeric pad</t>
+          <t>Wrong-tone typo surfaces intended word</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>inspect char keys</t>
+          <t>composing=ngưới</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>every char key is a digit; no letters/punctuation</t>
+          <t>bar contains người</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>NumericLayoutTest (unit)</t>
+          <t>TrigramFuzzyTest</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -5862,33 +6114,33 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NUMPAD-3</t>
+          <t>VIAC-3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Only ABC/backspace/enter specials; no space</t>
+          <t>Missing/substitution char typo</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>inspect special keys</t>
+          <t>composing=nhs</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>specials subset {ABC,BACKSPACE,ENTER}; ABC+backspace present; no space key</t>
+          <t>bar contains nhà</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>NumericLayoutTest (unit)</t>
+          <t>TrigramFuzzyTest</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -5900,37 +6152,33 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NUMPAD-4</t>
+          <t>VIAC-4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OTP field opens number-only keypad (on-device)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>real OTP/PIN field (e.g. VNeID, or numberPassword field)</t>
-        </is>
-      </c>
+          <t>Exact prefix not displaced by fuzzy</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>focus an OTP field with DraftRight keyboard</t>
+          <t>composing=ng limit2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>shows 3-col digit grid (1-9, ABC 0 back enter); NOT the ?123 symbols layer</t>
+          <t>returns người,ngon (exacts only, no fuzzy)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>On-device manual</t>
+          <t>TrigramFuzzyTest</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -5942,32 +6190,28 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>NUMPAD-5</t>
+          <t>VIAC-5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ABC escapes back to letters</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>numeric field focused</t>
-        </is>
-      </c>
+          <t>Far typo (dist&gt;1) surfaces nothing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>tap ABC on numeric pad</t>
+          <t>composing=zzzz</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>returns to alpha QWERTY layer</t>
+          <t>empty candidate list</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>On-device manual</t>
+          <t>TrigramFuzzyTest</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">

</xml_diff>

<commit_message>
feat(#207): JP/ZH space-to-convert reading → top candidate (Phase 2)
Standard JP/ZH IMEs convert the reading on space (kana→kanji, pinyin→hanzi);
DraftRight committed the raw reading + a space instead. Add it.

- LanguagePack.convertsOnSpace declarative trait (default false); Japanese +
  Chinese override true. English/Vietnamese/Korean keep space literal (Hangul
  assembles directly, no conversion).
- onSpace: when a conversion pack has a live reading, commit the top candidate
  (replaces the marked composing region) with no trailing space (CJK). Empty
  buffer falls through to a normal space. One chokepoint (convertReadingOnSpace),
  gated on the pack trait so Latin/Telex/Hangul are untouched (no regression).

ConvertOnSpaceTest 2/0. Conversion flow is IME-level (on-device gate JPSP-3/4).
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -25,6 +25,7 @@
     <sheet name="KBD-VI-SUGGEST" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="KBD-NUMPAD" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="KBD-VI-AUTOCORRECT" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="KBD-JP-CONVERT" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6046,20 +6047,261 @@
           <t>Substitution typo surfaces correction</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>composing=nqon</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>candidate bar contains ngon (edit dist 1)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>TrigramFuzzyTest</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>VIAC-2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Wrong-tone typo surfaces intended word</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>composing=ngưới</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>bar contains người</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>TrigramFuzzyTest</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>VIAC-3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Missing/substitution char typo</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>composing=nhs</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>bar contains nhà</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>TrigramFuzzyTest</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>VIAC-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Exact prefix not displaced by fuzzy</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>composing=ng limit2</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>returns người,ngon (exacts only, no fuzzy)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>TrigramFuzzyTest</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>VIAC-5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Far typo (dist&gt;1) surfaces nothing</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>composing=zzzz</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>empty candidate list</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>TrigramFuzzyTest</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Verified by</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>JPSP-1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>JP/ZH packs convert on space</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>composing=nqon</t>
+          <t>inspect convertsOnSpace</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>candidate bar contains ngon (edit dist 1)</t>
+          <t>Japanese + Chinese = true</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>TrigramFuzzyTest</t>
+          <t>ConvertOnSpaceTest</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -6076,28 +6318,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>VIAC-2</t>
+          <t>JPSP-2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Wrong-tone typo surfaces intended word</t>
+          <t>EN/VI/KO keep space literal</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>composing=ngưới</t>
+          <t>inspect convertsOnSpace</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>bar contains người</t>
+          <t>English, Vietnamese, Korean = false</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TrigramFuzzyTest</t>
+          <t>ConvertOnSpaceTest</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -6114,33 +6356,37 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>VIAC-3</t>
+          <t>JPSP-3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Missing/substitution char typo</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>JP space converts kana-&gt;kanji (on-device)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Japanese pack active, kana in buffer</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>composing=nhs</t>
+          <t>type nihongo -&gt; にほんご, press space</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>bar contains nhà</t>
+          <t>commits 日本語 (top candidate), no trailing space</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TrigramFuzzyTest</t>
+          <t>On-device manual</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -6152,74 +6398,40 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>VIAC-4</t>
+          <t>JPSP-4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Exact prefix not displaced by fuzzy</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>JP space with empty buffer = normal space</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Japanese pack, empty buffer</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>composing=ng limit2</t>
+          <t>press space with no reading</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>returns người,ngon (exacts only, no fuzzy)</t>
+          <t>inserts a normal space</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>TrigramFuzzyTest</t>
+          <t>On-device manual</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
-        <is>
-          <t>Tan</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>VIAC-5</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Far typo (dist&gt;1) surfaces nothing</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>composing=zzzz</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>empty candidate list</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>TrigramFuzzyTest</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
         <is>
           <t>Tan</t>
         </is>

</xml_diff>

<commit_message>
test(#207): CJK cycling on-device verification cases (CJKCYC-6..9)
On-device VERIFIED on Samsung A52: kanji→かんじ, space→漢字(pending), space→幹事
(cycle), enter→幹事 committed no-newline. Backspace-cancel manual. Clears the
'held off develop' gate from the wip commit — safe to merge.
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -26,6 +26,7 @@
     <sheet name="KBD-NUMPAD" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="KBD-VI-AUTOCORRECT" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="KBD-JP-CONVERT" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="KBD-CJK-CYCLE" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6288,7 +6289,6 @@
           <t>JP/ZH packs convert on space</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>inspect convertsOnSpace</t>
@@ -6326,7 +6326,6 @@
           <t>EN/VI/KO keep space literal</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>inspect convertsOnSpace</t>
@@ -6943,6 +6942,268 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Verified by</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CJKCYC-1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ConversionCycle wraps candidates</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>advance past last</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>wraps to top; idle/empty safe</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ConversionCycleTest</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CJKCYC-6</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>JP space converts to top candidate (pending)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>JP active, かんじ composed</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>press space</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>field shows 漢字 underlined (marked, not committed)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>On-device VERIFIED</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CJKCYC-7</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Repeat space cycles candidates</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>pending 漢字</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>press space again</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>cycles to 幹事 (still marked)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>On-device VERIFIED</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CJKCYC-8</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Enter confirms current candidate, no newline</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>pending 幹事</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>press enter</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>commits 幹事 (no underline), no newline, bar cleared</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>On-device VERIFIED</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CJKCYC-9</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Backspace cancels back to reading</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>pending 漢字</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>press backspace</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>reverts to かんじ composing</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>On-device manual</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
feat(#211): Chinese initials abbreviation (nh→你好, bj→北京), both platforms
A word's syllable initials commit the whole word — a signature ZH speed feature.
Extends PinyinCandidateEngine: an initials index (bj → 北京) derived once from the
dictionary + PinyinSegmenter — no new source of truth (RULE #1), and Japanese
(same shared DictionaryCandidateEngine) stays untouched. Ranks below exact word
and segmented sentence, above the raw fallback.

Tests: PinyinCandidateEngine 8/0 on each platform.
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -7210,7 +7210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7266,7 +7266,6 @@
           <t>Segment two-syllable pinyin</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>segment(woshi)</t>
@@ -7304,7 +7303,6 @@
           <t>Prefer longest syllable</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>segment(xianggang)</t>
@@ -7342,7 +7340,6 @@
           <t>Backtrack on bad greedy pick</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>segment(xier)</t>
@@ -7380,7 +7377,6 @@
           <t>Run-together pinyin -&gt; segmented hanzi candidate</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>suggest(woshi)</t>
@@ -7418,7 +7414,6 @@
           <t>Exact word ranks above segmented</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>suggest(nihao)</t>
@@ -7456,7 +7451,6 @@
           <t>Syllable set parity Android&lt;-&gt;iOS</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>run check-pinyin-syllables-parity.py</t>
@@ -7520,6 +7514,86 @@
         </is>
       </c>
       <c r="H8" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ZHPY-13</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Initials abbreviation -&gt; whole word</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>suggest(nh) / suggest(bj)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>你好 / 北京 in candidates</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PinyinCandidateEngine(Test) x2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ZHPY-14</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>On-device abbreviation</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>中文 enabled</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>type nh</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>你好 appears in candidate bar</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>On-device</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>Tan</t>
         </is>

</xml_diff>

<commit_message>
feat(#211): fuzzy pinyin (zh=z, ch=c, sh=s, ang=an…), both platforms
A sloppy spelling still finds the word — "zongguo" → 中国, "si" → 是. PinyinFuzzy
folds retroflex↔dental initials + nasal finals; PinyinCandidateEngine builds a
folded index from the dictionary (no new source of truth — RULE #1) and adds
fuzzy matches to the derived candidates. Japanese untouched.

Tests: PinyinFuzzy 3/0 + PinyinCandidateEngine 9/0 each platform.
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -7210,7 +7210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7530,7 +7530,6 @@
           <t>Initials abbreviation -&gt; whole word</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>suggest(nh) / suggest(bj)</t>
@@ -7594,6 +7593,124 @@
         </is>
       </c>
       <c r="H10" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ZHPY-15</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Fuzzy pinyin fold (zh=z, ing=in...)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>fold(shi)=si, fold(zhongguo)=zongguo</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>folds retroflex/nasal</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>PinyinFuzzy(Test) x2</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ZHPY-16</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Fuzzy match finds word</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>suggest(si) / suggest(zongguo)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>是 / 中国 in candidates</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PinyinCandidateEngine(Test) x2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ZHPY-17</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>On-device fuzzy</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>中文</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>type si</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>是 appears in candidate bar</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>On-device</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>Tan</t>
         </is>

</xml_diff>

<commit_message>
feat(#212): JP flick core — kana map + gesture resolution (phase 1)
The pure, testable heart of フリック input (both platforms):
- FlickGesture.resolve(dx,dy,threshold) → TAP/LEFT/UP/RIGHT/DOWN (screen coords).
- FlickLayout: the 12-key gojūon kana map (tap=あ, ←=い, ↑=う, →=え, ↓=お; や/わ
  specials). One cited linguistic source, mirrored Kotlin↔Swift.
- scripts/check-flick-layout-parity.py: 48 (row,dir,kana) entries must agree
  across platforms; wired into the mobile-parity CI job.

Tests: FlickTest 4/0 each platform. These primitives are consumed by the flick
keyboard VIEW + IME wiring (#212 phase 2, device) and iOS view (phase 4) — public
API awaiting those disclosed follow-ups, not dead code.
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -28,6 +28,7 @@
     <sheet name="KBD-JP-CONVERT" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="KBD-CJK-CYCLE" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="KBD-ZH-PINYIN" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="KBD-JP-FLICK" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -7609,7 +7610,6 @@
           <t>Fuzzy pinyin fold (zh=z, ing=in...)</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>fold(shi)=si, fold(zhongguo)=zongguo</t>
@@ -7647,7 +7647,6 @@
           <t>Fuzzy match finds word</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
           <t>suggest(si) / suggest(zongguo)</t>
@@ -7711,6 +7710,252 @@
         </is>
       </c>
       <c r="H13" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TC-ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Verified by</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>JPFLICK-1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Small movement = tap</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>resolve(0,0) / resolve(10,-12)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>TAP</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>FlickTest(s)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>JPFLICK-2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Flick resolves by dominant axis</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>resolve(-100,5)/(100,-5)/(5,-100)/(-5,100)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>LEFT/RIGHT/UP/DOWN</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>FlickTest(s)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>JPFLICK-3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Uniform gojuon rows map vowels</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>kanaFor(あ,LEFT) etc</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>い/こ/つ/せ; tap=head</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>FlickTest(s)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>JPFLICK-4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Special rows や/わ</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>kanaFor(や,UP)/(わ,UP)/(わ,LEFT)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ゆ/ん/を; や LEFT null</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>FlickTest(s)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>JPFLICK-5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Flick kana map parity Android&lt;-&gt;iOS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>run check-flick-layout-parity.py</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>48 entries agree</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>CI parity guard</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>Tan</t>
         </is>

</xml_diff>

<commit_message>
docs: VIAC-6..13 test cases for auto-correct-on-space + undo (#207)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -5994,7 +5994,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6219,6 +6219,337 @@
         </is>
       </c>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>VIAC-6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Space auto-corrects one-edit typo</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>type khoog (khôg), press space</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>field shows "không " (corrected + space)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>AutoCorrectorVectorsTest/Tests + device 2026-09-03</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>VIAC-7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Leading capital preserved on correction</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>VI pack, auto-caps on</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>type Khôg, space</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>"Không " — capital carried over</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>AutoCorrectorVectorsTest/Tests + device 2026-09-03</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>VIAC-8</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Backspace right after correction restores typed word</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>VIAC-6 done</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>press backspace once</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>field shows "khôg " again</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>device 2026-09-03</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>VIAC-9</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Undo is one-shot</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>VIAC-8 done</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>press backspace again</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>plain delete (space removed), no second revert</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>AutoCorrectUndoTest/Tests + device 2026-09-03</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>VIAC-10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Real word never corrected</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>VI pack active</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>type anh, space</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>"anh " untouched</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>AutoCorrectorVectorsTest/Tests + device 2026-09-03</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>VIAC-11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ALL-CAPS / mixed case left alone</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>type KHÔG or kHôg, space</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>committed as typed</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>AutoCorrectorVectorsTest/Tests</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>VIAC-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Stale field (#71 Zalo clear) not auto-corrected</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>app clears field silently before space</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>send msg in Zalo, press space in empty field</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>no resurrection of sent word; guard drops stale buffer</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>code review 8e49d9ae; manual Zalo check pending</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>VIAC-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Stale undo disarmed after more typing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>correction armed, keep typing, retype "không "</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>backspace after the retyped word</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>plain delete — earlier undo must NOT swap word to old typo</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>AutoCorrectUndoTest isLive + lifecycle disarms</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>Tan</t>
         </is>
@@ -7782,7 +8113,6 @@
           <t>Small movement = tap</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
           <t>resolve(0,0) / resolve(10,-12)</t>
@@ -7820,7 +8150,6 @@
           <t>Flick resolves by dominant axis</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>resolve(-100,5)/(100,-5)/(5,-100)/(-5,100)</t>
@@ -7858,7 +8187,6 @@
           <t>Uniform gojuon rows map vowels</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>kanaFor(あ,LEFT) etc</t>
@@ -7896,7 +8224,6 @@
           <t>Special rows や/わ</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
           <t>kanaFor(や,UP)/(わ,UP)/(わ,LEFT)</t>
@@ -7934,7 +8261,6 @@
           <t>Flick kana map parity Android&lt;-&gt;iOS</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
           <t>run check-flick-layout-parity.py</t>

</xml_diff>